<commit_message>
snapshot b31b95933: release(b4): prepare 0.11.51 ow-92 with measured residuals and verified economy
Source-Commit: b31b959334bc51dff009b3f711c0d0b44536a571
</commit_message>
<xml_diff>
--- a/open-world/config/excel/任务.xlsx
+++ b/open-world/config/excel/任务.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="Rb384e06b98c844cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导出" sheetId="2" r:id="Rd6f9310fd5f547da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务类型" sheetId="3" r:id="R648a6ef2f61447fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务" sheetId="4" r:id="Rcfb9dd9f6eaa419b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步骤" sheetId="5" r:id="Rce88293f0a8246a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路线" sheetId="6" r:id="R9bd6ca3db4bb4a1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="条件" sheetId="7" r:id="R202ae1e0a74a403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传闻" sheetId="8" r:id="R79aaad4a6ae94d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技能找回" sheetId="9" r:id="Rbd709e079a2a4a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R964649ce2c614870"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导出" sheetId="2" r:id="R7038dbc906af4176"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务类型" sheetId="3" r:id="R706936ad85ca462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务" sheetId="4" r:id="R427c11d2138441eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步骤" sheetId="5" r:id="Ra13f9c8839864296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路线" sheetId="6" r:id="R49a2f2f16377427e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="条件" sheetId="7" r:id="R6fe00d1fc6bf408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="传闻" sheetId="8" r:id="R9cc16a9c92a84e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技能找回" sheetId="9" r:id="Ra4d1caae2bb74624"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,6 +174,7 @@
     <x:author>tc={8B21994E-F85D-4295-A3A0-3E11128245CD}</x:author>
     <x:author>tc={5F050F4B-784D-45ED-9CCE-541796FF516C}</x:author>
     <x:author/>
+    <x:author>tc={11A5B88D-5B8D-44D6-A2A7-40E93B8D413E}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="A1" authorId="0">
@@ -553,6 +554,16 @@
       <x:text>
         <x:r>
           <x:t>D12：任务完成发放的回响碎片数量，仅一次。</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="BC2" authorId="12">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    首通结算的T1材料，JSON {materialId:非负整数个数}。关口预算记录绑定hub_node且hub_return=true/journal=false：不接取、不展示任务，由现有节点首通事实一次性结算，不参与本日×2。 唯一源：config/excel 工作簿；经 pnpm config:export 导出，服务端消费。数值来自经审核的 B4 推导计划，不在运行时另设第二份配置。</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -1316,6 +1327,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:person displayName="HUB 配置字段说明" id="{647D2B22-8B16-4115-BD1B-35B9123D397F}"/>
   <xltc:person displayName="tc={094C4E01-3C4C-4447-82A0-FC4FC1A64DCE}" id="{BEFC62CC-411B-A519-36CC-702EF782B778}"/>
   <xltc:person displayName="tc={BF0E8B7E-C8A2-4328-8E42-B20C885C90EE}" id="{A92C1EAE-7AD0-8E1F-762C-433E02D8E1A0}"/>
   <xltc:person displayName="None" id="{A526D1F0-D2D1-FEBE-9CEF-436996D68996}"/>
@@ -1567,6 +1579,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="BC2" dT="2026-10-22T16:19:42.898" personId="{647D2B22-8B16-4115-BD1B-35B9123D397F}" id="{11A5B88D-5B8D-44D6-A2A7-40E93B8D413E}">
+    <xltc:text>首通结算的T1材料，JSON {materialId:非负整数个数}。关口预算记录绑定hub_node且hub_return=true/journal=false：不接取、不展示任务，由现有节点首通事实一次性结算，不参与本日×2。 唯一源：config/excel 工作簿；经 pnpm config:export 导出，服务端消费。数值来自经审核的 B4 推导计划，不在运行时另设第二份配置。</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1905,7 +1925,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe9f7e8eda31480f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc7e971848454d16"/>
 </x:worksheet>
 </file>
 
@@ -2317,7 +2337,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7437344fc7ab4e1a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35d63bf1b1334097"/>
 </x:worksheet>
 </file>
 
@@ -2375,6 +2395,7 @@
     <x:col min="48" max="48" width="24" hidden="0" customWidth="1"/>
     <x:col min="49" max="49" width="24" hidden="0" customWidth="1"/>
     <x:col min="50" max="50" width="24" hidden="0" customWidth="1"/>
+    <x:col min="55" max="55" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2628,6 +2649,9 @@
       <x:c r="BB1" t="str">
         <x:v>hub_commission</x:v>
       </x:c>
+      <x:c r="BC1" t="str">
+        <x:v>reward_materials</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="inlineStr">
@@ -2880,6 +2904,9 @@
       <x:c r="BB2" t="str">
         <x:v>hub_commission</x:v>
       </x:c>
+      <x:c r="BC2" t="str">
+        <x:v>reward_materials</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="inlineStr">
@@ -3131,6 +3158,9 @@
       </x:c>
       <x:c r="BB3" t="str">
         <x:v>bool</x:v>
+      </x:c>
+      <x:c r="BC3" t="str">
+        <x:v>json</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -31353,7 +31383,9 @@
       <x:c r="AV317"/>
       <x:c r="AW317"/>
       <x:c r="AX317"/>
-      <x:c r="AY317"/>
+      <x:c r="AY317" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="AZ317"/>
       <x:c r="BA317"/>
       <x:c r="BB317"/>
@@ -31441,7 +31473,9 @@
       <x:c r="AV318"/>
       <x:c r="AW318"/>
       <x:c r="AX318"/>
-      <x:c r="AY318"/>
+      <x:c r="AY318" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="AZ318"/>
       <x:c r="BA318"/>
       <x:c r="BB318"/>
@@ -31529,7 +31563,9 @@
       <x:c r="AV319"/>
       <x:c r="AW319"/>
       <x:c r="AX319"/>
-      <x:c r="AY319"/>
+      <x:c r="AY319" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="AZ319"/>
       <x:c r="BA319"/>
       <x:c r="BB319"/>
@@ -31617,7 +31653,9 @@
       <x:c r="AV320"/>
       <x:c r="AW320"/>
       <x:c r="AX320"/>
-      <x:c r="AY320"/>
+      <x:c r="AY320" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="AZ320"/>
       <x:c r="BA320"/>
       <x:c r="BB320"/>
@@ -31705,14 +31743,210 @@
       <x:c r="AV321"/>
       <x:c r="AW321"/>
       <x:c r="AX321"/>
-      <x:c r="AY321"/>
+      <x:c r="AY321" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="AZ321"/>
       <x:c r="BA321"/>
       <x:c r="BB321"/>
     </x:row>
+    <x:row r="322">
+      <x:c r="A322" t="str">
+        <x:v>hub-gate-reward-wind</x:v>
+      </x:c>
+      <x:c r="B322" t="str">
+        <x:v>starsea</x:v>
+      </x:c>
+      <x:c r="C322" t="str">
+        <x:v>ss-c01</x:v>
+      </x:c>
+      <x:c r="D322" t="n">
+        <x:v>9004</x:v>
+      </x:c>
+      <x:c r="E322" t="str">
+        <x:v>side</x:v>
+      </x:c>
+      <x:c r="F322" t="str">
+        <x:v>击退登港先锋首通奖励</x:v>
+      </x:c>
+      <x:c r="G322" t="str">
+        <x:v>击退登港先锋首通奖励</x:v>
+      </x:c>
+      <x:c r="H322"/>
+      <x:c r="I322" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="J322"/>
+      <x:c r="K322" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="L322"/>
+      <x:c r="M322"/>
+      <x:c r="N322"/>
+      <x:c r="O322"/>
+      <x:c r="P322"/>
+      <x:c r="Q322"/>
+      <x:c r="R322"/>
+      <x:c r="S322"/>
+      <x:c r="T322" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U322" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V322" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W322" s="14" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X322"/>
+      <x:c r="Y322"/>
+      <x:c r="Z322"/>
+      <x:c r="AA322"/>
+      <x:c r="AB322"/>
+      <x:c r="AC322"/>
+      <x:c r="AD322"/>
+      <x:c r="AE322"/>
+      <x:c r="AF322"/>
+      <x:c r="AG322" t="str">
+        <x:v>["首通结算"]</x:v>
+      </x:c>
+      <x:c r="AH322"/>
+      <x:c r="AI322"/>
+      <x:c r="AJ322"/>
+      <x:c r="AK322"/>
+      <x:c r="AL322" t="str">
+        <x:v>hub-first-clear-reward</x:v>
+      </x:c>
+      <x:c r="AM322"/>
+      <x:c r="AN322"/>
+      <x:c r="AO322"/>
+      <x:c r="AP322"/>
+      <x:c r="AQ322"/>
+      <x:c r="AR322" s="14" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS322"/>
+      <x:c r="AT322"/>
+      <x:c r="AU322"/>
+      <x:c r="AV322"/>
+      <x:c r="AW322"/>
+      <x:c r="AX322"/>
+      <x:c r="AY322" s="14" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AZ322" t="str">
+        <x:v>wind-gate</x:v>
+      </x:c>
+      <x:c r="BA322" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB322"/>
+      <x:c r="BC322" t="str">
+        <x:v>{"wind_ore":4,"wind_herb":4}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323">
+      <x:c r="A323" t="str">
+        <x:v>hub-gate-reward-mist</x:v>
+      </x:c>
+      <x:c r="B323" t="str">
+        <x:v>starsea</x:v>
+      </x:c>
+      <x:c r="C323" t="str">
+        <x:v>ss-c02</x:v>
+      </x:c>
+      <x:c r="D323" t="n">
+        <x:v>9005</x:v>
+      </x:c>
+      <x:c r="E323" t="str">
+        <x:v>side</x:v>
+      </x:c>
+      <x:c r="F323" t="str">
+        <x:v>截击军需官首通奖励</x:v>
+      </x:c>
+      <x:c r="G323" t="str">
+        <x:v>截击军需官首通奖励</x:v>
+      </x:c>
+      <x:c r="H323"/>
+      <x:c r="I323" t="str">
+        <x:v>ss-npc-qingmang</x:v>
+      </x:c>
+      <x:c r="J323"/>
+      <x:c r="K323" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="L323"/>
+      <x:c r="M323"/>
+      <x:c r="N323"/>
+      <x:c r="O323"/>
+      <x:c r="P323"/>
+      <x:c r="Q323"/>
+      <x:c r="R323"/>
+      <x:c r="S323"/>
+      <x:c r="T323" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U323" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V323" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W323" s="14" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X323"/>
+      <x:c r="Y323"/>
+      <x:c r="Z323"/>
+      <x:c r="AA323"/>
+      <x:c r="AB323"/>
+      <x:c r="AC323"/>
+      <x:c r="AD323"/>
+      <x:c r="AE323"/>
+      <x:c r="AF323"/>
+      <x:c r="AG323" t="str">
+        <x:v>["首通结算"]</x:v>
+      </x:c>
+      <x:c r="AH323"/>
+      <x:c r="AI323"/>
+      <x:c r="AJ323"/>
+      <x:c r="AK323"/>
+      <x:c r="AL323" t="str">
+        <x:v>hub-first-clear-reward</x:v>
+      </x:c>
+      <x:c r="AM323"/>
+      <x:c r="AN323"/>
+      <x:c r="AO323"/>
+      <x:c r="AP323"/>
+      <x:c r="AQ323"/>
+      <x:c r="AR323" s="14" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS323"/>
+      <x:c r="AT323"/>
+      <x:c r="AU323"/>
+      <x:c r="AV323"/>
+      <x:c r="AW323"/>
+      <x:c r="AX323"/>
+      <x:c r="AY323" s="14" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AZ323" t="str">
+        <x:v>mist-gate</x:v>
+      </x:c>
+      <x:c r="BA323" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB323"/>
+      <x:c r="BC323" t="str">
+        <x:v>{"mist_ore":6,"mist_herb":6}</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ec7fcc6907244f8"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7ce9c34d249be"/>
 </x:worksheet>
 </file>
 
@@ -50623,9 +50857,105 @@
       <x:c r="AC393"/>
       <x:c r="AD393"/>
     </x:row>
+    <x:row r="394">
+      <x:c r="A394" t="str">
+        <x:v>hub-gate-reward-wind</x:v>
+      </x:c>
+      <x:c r="B394" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C394" t="str">
+        <x:v>hub_fact</x:v>
+      </x:c>
+      <x:c r="D394" t="str">
+        <x:v>hub-node:wind-gate</x:v>
+      </x:c>
+      <x:c r="E394"/>
+      <x:c r="F394" t="str">
+        <x:v>击退登港先锋首通奖励</x:v>
+      </x:c>
+      <x:c r="G394"/>
+      <x:c r="H394" t="str">
+        <x:v>ss-map-port</x:v>
+      </x:c>
+      <x:c r="I394" t="str">
+        <x:v>stargate</x:v>
+      </x:c>
+      <x:c r="J394"/>
+      <x:c r="K394"/>
+      <x:c r="L394"/>
+      <x:c r="M394"/>
+      <x:c r="N394"/>
+      <x:c r="O394"/>
+      <x:c r="P394"/>
+      <x:c r="Q394"/>
+      <x:c r="R394"/>
+      <x:c r="S394"/>
+      <x:c r="T394"/>
+      <x:c r="U394"/>
+      <x:c r="V394"/>
+      <x:c r="W394"/>
+      <x:c r="X394"/>
+      <x:c r="Y394" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z394"/>
+      <x:c r="AA394"/>
+      <x:c r="AB394"/>
+      <x:c r="AC394"/>
+      <x:c r="AD394"/>
+    </x:row>
+    <x:row r="395">
+      <x:c r="A395" t="str">
+        <x:v>hub-gate-reward-mist</x:v>
+      </x:c>
+      <x:c r="B395" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C395" t="str">
+        <x:v>hub_fact</x:v>
+      </x:c>
+      <x:c r="D395" t="str">
+        <x:v>hub-node:mist-gate</x:v>
+      </x:c>
+      <x:c r="E395"/>
+      <x:c r="F395" t="str">
+        <x:v>截击军需官首通奖励</x:v>
+      </x:c>
+      <x:c r="G395"/>
+      <x:c r="H395" t="str">
+        <x:v>ss-map-port</x:v>
+      </x:c>
+      <x:c r="I395" t="str">
+        <x:v>stargate</x:v>
+      </x:c>
+      <x:c r="J395"/>
+      <x:c r="K395"/>
+      <x:c r="L395"/>
+      <x:c r="M395"/>
+      <x:c r="N395"/>
+      <x:c r="O395"/>
+      <x:c r="P395"/>
+      <x:c r="Q395"/>
+      <x:c r="R395"/>
+      <x:c r="S395"/>
+      <x:c r="T395"/>
+      <x:c r="U395"/>
+      <x:c r="V395"/>
+      <x:c r="W395"/>
+      <x:c r="X395"/>
+      <x:c r="Y395" s="14" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z395"/>
+      <x:c r="AA395"/>
+      <x:c r="AB395"/>
+      <x:c r="AC395"/>
+      <x:c r="AD395"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51087d28e87043e9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26aa3475b07b4d4f"/>
 </x:worksheet>
 </file>
 
@@ -51691,7 +52021,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R745f11af0cc44127"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9386d05a02f5473b"/>
 </x:worksheet>
 </file>
 
@@ -69278,7 +69608,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e6ec6deeea24a1f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d39cf7fae2d4c39"/>
 </x:worksheet>
 </file>
 
@@ -70074,7 +70404,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ccd1f50e5744c5e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25c1ad360fda4200"/>
 </x:worksheet>
 </file>
 
@@ -70975,6 +71305,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8463ef2ba35746cd"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c67c728aa0141e9"/>
 </x:worksheet>
 </file>
</xml_diff>